<commit_message>
Updated Rosters and teams
</commit_message>
<xml_diff>
--- a/game-stats/Week1_Desert-Lions_vs_K2.xlsx
+++ b/game-stats/Week1_Desert-Lions_vs_K2.xlsx
@@ -522,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1147,7 +1147,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Mostafa El-leboudi</t>
+          <t>Mostafa El-Leboudi</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -1177,6 +1177,123 @@
         <v>0</v>
       </c>
       <c r="K16" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Shafiq Said</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>WR/DB</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Ahmad Ashkar</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>OL/DL</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Osama Alowaid</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>WR/DL</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1734,16 +1851,16 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
-        <v>88</v>
+        <v>3</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Mohammed Aqrabawi</t>
+          <t>Ahmad Jaffal</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>DL/WR</t>
+          <t>DL</t>
         </is>
       </c>
       <c r="D14" s="4" t="n">
@@ -1773,16 +1890,16 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Ahmad Jaffal</t>
+          <t>Ibrahim Ahmed</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>DL</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="D15" s="4" t="n">
@@ -1812,16 +1929,16 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Ibrahim Ahmed</t>
+          <t>Yusuf Saleh</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>DB/WR</t>
         </is>
       </c>
       <c r="D16" s="4" t="n">
@@ -1851,16 +1968,16 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Yusuf Saleh</t>
+          <t>Aleem Abdulla</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>DB/WR</t>
+          <t>S/RB</t>
         </is>
       </c>
       <c r="D17" s="4" t="n">
@@ -1890,16 +2007,16 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Aleem Abdulla</t>
+          <t>Jooma Abderazzaq</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>S/RB</t>
+          <t>OL/DL</t>
         </is>
       </c>
       <c r="D18" s="4" t="n">

</xml_diff>